<commit_message>
Updated NGA model - 2025-12-12 15:29
</commit_message>
<xml_diff>
--- a/VerveStacks_NGA/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_NGA/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr updateLinks="never"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4C48DD9-DED7-479B-A74E-1DB16C47A208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E9D28A6-5A63-4F06-8140-582408A00B6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28702" yWindow="-98" windowWidth="28995" windowHeight="15675" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AVA" sheetId="6" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="84">
   <si>
     <t>PSET_PN</t>
   </si>
@@ -263,6 +263,33 @@
   </si>
   <si>
     <t>ELC_wo*</t>
+  </si>
+  <si>
+    <t>pset_set</t>
+  </si>
+  <si>
+    <t>limtype</t>
+  </si>
+  <si>
+    <t>other_indexes</t>
+  </si>
+  <si>
+    <t>flo_emis</t>
+  </si>
+  <si>
+    <t>gas</t>
+  </si>
+  <si>
+    <t>co2</t>
+  </si>
+  <si>
+    <t>co2captured</t>
+  </si>
+  <si>
+    <t>*ccs*</t>
+  </si>
+  <si>
+    <t>coal,oil,bioenergy</t>
   </si>
 </sst>
 </file>
@@ -1257,7 +1284,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="C4:X50"/>
+  <dimension ref="C4:X57"/>
   <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="13.3984375" bestFit="1" customWidth="1"/>
@@ -2008,7 +2035,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="49" spans="3:6" x14ac:dyDescent="0.45">
+    <row r="49" spans="3:13" x14ac:dyDescent="0.45">
       <c r="C49" t="s">
         <v>64</v>
       </c>
@@ -2022,7 +2049,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="50" spans="3:6" x14ac:dyDescent="0.45">
+    <row r="50" spans="3:13" x14ac:dyDescent="0.45">
       <c r="C50" t="s">
         <v>69</v>
       </c>
@@ -2034,6 +2061,86 @@
       </c>
       <c r="F50" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="54" spans="3:13" x14ac:dyDescent="0.45">
+      <c r="C54" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" spans="3:13" x14ac:dyDescent="0.45">
+      <c r="C55" t="s">
+        <v>25</v>
+      </c>
+      <c r="D55" t="s">
+        <v>75</v>
+      </c>
+      <c r="E55" t="s">
+        <v>65</v>
+      </c>
+      <c r="F55" t="s">
+        <v>21</v>
+      </c>
+      <c r="G55" t="s">
+        <v>66</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55">
+        <v>2022</v>
+      </c>
+      <c r="J55">
+        <v>2030</v>
+      </c>
+      <c r="K55" t="s">
+        <v>76</v>
+      </c>
+      <c r="L55" t="s">
+        <v>77</v>
+      </c>
+      <c r="M55" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="56" spans="3:13" x14ac:dyDescent="0.45">
+      <c r="C56" t="s">
+        <v>78</v>
+      </c>
+      <c r="E56" t="s">
+        <v>79</v>
+      </c>
+      <c r="F56" t="s">
+        <v>82</v>
+      </c>
+      <c r="I56">
+        <v>0.95</v>
+      </c>
+      <c r="L56" t="s">
+        <v>80</v>
+      </c>
+      <c r="M56" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="57" spans="3:13" x14ac:dyDescent="0.45">
+      <c r="C57" t="s">
+        <v>78</v>
+      </c>
+      <c r="E57" t="s">
+        <v>83</v>
+      </c>
+      <c r="F57" t="s">
+        <v>82</v>
+      </c>
+      <c r="I57">
+        <v>0.85</v>
+      </c>
+      <c r="L57" t="s">
+        <v>80</v>
+      </c>
+      <c r="M57" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>